<commit_message>
excel and xml generator modified
</commit_message>
<xml_diff>
--- a/dra_metadata.xlsx
+++ b/dra_metadata.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10536" tabRatio="430"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="24288" windowHeight="8952" tabRatio="430"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="9" r:id="rId1"/>
@@ -65,7 +65,9 @@
             <family val="3"/>
             <charset val="128"/>
           </rPr>
-          <t>YYYY-MM-DD (e.g, 2024-01-01)</t>
+          <t>YYYY-MM-DD (e.g, 2024-01-01)
+For immediate release, 
+enter date of submission.</t>
         </r>
       </text>
     </comment>
@@ -565,10 +567,6 @@
     <t>AB 310 Genetic Analyzer</t>
   </si>
   <si>
-    <t>v1.0</t>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>cDNA_randomPriming</t>
   </si>
   <si>
@@ -741,12 +739,16 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>2020-04-08 Bioinformation and DDBJ Center</t>
+    <t>This excel file is used to generate Submission, Experiment and Run XMLs for DDBJ Sequence Read Archive (DRA) submission. 
+Please see https://github.com/ddbj/submission-excel2xml for details.</t>
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>This excel file is used to generate Submission, Experiment and Run XMLs for DDBJ Sequence Read Archive (DRA) submission. 
-Please see https://github.com/ddbj/submission-excel2xml for details.</t>
+    <t>v1.1</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>2020-10-09 Bioinformation and DDBJ Center</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -1225,27 +1227,27 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="5" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="5" t="s">
-        <v>109</v>
-      </c>
-    </row>
     <row r="4" spans="1:1" ht="26.4">
       <c r="A4" s="7" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="16" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="18" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>
@@ -1271,24 +1273,24 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="C1" s="17" t="s">
         <v>134</v>
       </c>
-      <c r="B1" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="C1" s="17" t="s">
+    </row>
+    <row r="2" spans="1:3">
+      <c r="C2" s="3"/>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="16" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="C2" s="3"/>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="16" t="s">
+      <c r="B4" s="16" t="s">
         <v>136</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1330,7 +1332,7 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="16" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1" s="16" t="s">
         <v>9</v>
@@ -1426,7 +1428,7 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="16" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1" s="16" t="s">
         <v>9</v>
@@ -1460,7 +1462,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C1" s="17" t="s">
         <v>6</v>
@@ -27926,7 +27928,7 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B3" s="11" t="s">
         <v>28</v>
@@ -27938,7 +27940,7 @@
         <v>30</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>8</v>
@@ -27951,7 +27953,7 @@
         <v>27</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>33</v>
@@ -27970,7 +27972,7 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>37</v>
@@ -27983,7 +27985,7 @@
       </c>
       <c r="E5" s="10"/>
       <c r="F5" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G5" s="10"/>
       <c r="H5" s="10"/>
@@ -27996,7 +27998,7 @@
         <v>41</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>43</v>
@@ -28033,10 +28035,10 @@
         <v>40</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>48</v>
@@ -28050,10 +28052,10 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="10" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>72</v>
@@ -28063,7 +28065,7 @@
       </c>
       <c r="E9" s="10"/>
       <c r="F9" s="10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G9" s="10"/>
       <c r="H9" s="10"/>
@@ -28092,7 +28094,7 @@
         <v>55</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>64</v>
@@ -28105,10 +28107,10 @@
     <row r="12" spans="1:8">
       <c r="A12" s="13"/>
       <c r="B12" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>19</v>
@@ -28121,7 +28123,7 @@
     <row r="13" spans="1:8">
       <c r="A13" s="10"/>
       <c r="B13" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>47</v>
@@ -28137,10 +28139,10 @@
     <row r="14" spans="1:8">
       <c r="A14" s="10"/>
       <c r="B14" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>57</v>
@@ -28153,13 +28155,13 @@
     <row r="15" spans="1:8">
       <c r="A15" s="10"/>
       <c r="B15" s="11" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C15" s="10" t="s">
         <v>49</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
@@ -28169,13 +28171,13 @@
     <row r="16" spans="1:8">
       <c r="A16" s="10"/>
       <c r="B16" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C16" s="10" t="s">
         <v>53</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
@@ -28191,7 +28193,7 @@
         <v>56</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
@@ -28217,7 +28219,7 @@
     <row r="19" spans="1:8">
       <c r="A19" s="10"/>
       <c r="B19" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C19" s="10" t="s">
         <v>62</v>
@@ -28233,13 +28235,13 @@
     <row r="20" spans="1:8">
       <c r="A20" s="10"/>
       <c r="B20" s="11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C20" s="10" t="s">
         <v>63</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
@@ -28249,7 +28251,7 @@
     <row r="21" spans="1:8">
       <c r="A21" s="10"/>
       <c r="B21" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C21" s="10" t="s">
         <v>65</v>
@@ -28265,13 +28267,13 @@
     <row r="22" spans="1:8">
       <c r="A22" s="10"/>
       <c r="B22" s="11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C22" s="10" t="s">
         <v>67</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
@@ -28281,13 +28283,13 @@
     <row r="23" spans="1:8">
       <c r="A23" s="10"/>
       <c r="B23" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C23" s="10" t="s">
         <v>4</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
@@ -28297,7 +28299,7 @@
     <row r="24" spans="1:8">
       <c r="A24" s="10"/>
       <c r="B24" s="11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C24" s="10" t="s">
         <v>75</v>
@@ -28319,7 +28321,7 @@
         <v>78</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
@@ -28361,7 +28363,7 @@
     <row r="28" spans="1:8">
       <c r="A28" s="10"/>
       <c r="B28" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C28" s="10" t="s">
         <v>86</v>
@@ -28380,7 +28382,7 @@
         <v>85</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D29" s="10" t="s">
         <v>82</v>
@@ -28452,10 +28454,10 @@
       <c r="A34" s="10"/>
       <c r="B34" s="11"/>
       <c r="C34" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
@@ -28466,10 +28468,10 @@
       <c r="A35" s="10"/>
       <c r="B35" s="11"/>
       <c r="C35" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
@@ -28480,10 +28482,10 @@
       <c r="A36" s="10"/>
       <c r="B36" s="11"/>
       <c r="C36" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E36" s="10"/>
       <c r="F36" s="10"/>
@@ -28533,7 +28535,7 @@
       <c r="B40" s="11"/>
       <c r="C40" s="10"/>
       <c r="D40" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E40" s="10"/>
       <c r="F40" s="10"/>
@@ -28552,12 +28554,12 @@
     </row>
     <row r="43" spans="1:8">
       <c r="D43" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="44" spans="1:8">
       <c r="D44" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -28607,7 +28609,7 @@
     </row>
     <row r="54" spans="4:4">
       <c r="D54" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="55" spans="4:4">

</xml_diff>

<commit_message>
update to xsd 1.5.9
</commit_message>
<xml_diff>
--- a/dra_metadata.xlsx
+++ b/dra_metadata.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.112.22\ykodama\github\submission-excel2xml\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\ddbjs4.nig.ac.jp\ykodama\github\submission-excel2xml\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="11820" tabRatio="430"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20124" windowHeight="8772" tabRatio="430"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="9" r:id="rId1"/>
@@ -256,7 +256,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="178">
   <si>
     <t>Library Source</t>
   </si>
@@ -280,9 +280,6 @@
   </si>
   <si>
     <t>MD5 Checksum</t>
-  </si>
-  <si>
-    <t>fastq</t>
   </si>
   <si>
     <t>Title</t>
@@ -728,16 +725,10 @@
     <t>Restriction Digest</t>
   </si>
   <si>
-    <t xml:space="preserve">Illumina MiniSeq      </t>
-  </si>
-  <si>
     <t>5-methylcytidine antibody</t>
   </si>
   <si>
     <t>MBD2 protein methyl-CpG binding domain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NextSeq 550            </t>
   </si>
   <si>
     <t>padlock probes capture method</t>
@@ -762,16 +753,59 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>v1.1</t>
+    <t>BioProject accession</t>
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>2020-11-11 Bioinformation and DDBJ Center</t>
+    <t>2021-07-13 Bioinformation and DDBJ Center</t>
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>BioProject accession</t>
+    <t>v1.2</t>
     <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>NOMe-Seq</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>NextSeq 1000</t>
+  </si>
+  <si>
+    <t>NextSeq 2000</t>
+  </si>
+  <si>
+    <t>NextSeq 550</t>
+  </si>
+  <si>
+    <t>BGISEQ-500</t>
+  </si>
+  <si>
+    <t>DNBSEQ-G400</t>
+  </si>
+  <si>
+    <t>DNBSEQ-T7</t>
+  </si>
+  <si>
+    <t>DNBSEQ-G50</t>
+  </si>
+  <si>
+    <t>MGISEQ-2000RS</t>
+  </si>
+  <si>
+    <t>Sequel II</t>
+  </si>
+  <si>
+    <t>Ion GeneStudio S5</t>
+  </si>
+  <si>
+    <t>Ion GeneStudio S5 plus</t>
+  </si>
+  <si>
+    <t>Ion GeneStudio S5 prime</t>
+  </si>
+  <si>
+    <t>Illumina MiniSeq</t>
   </si>
 </sst>
 </file>
@@ -1249,27 +1283,27 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="5" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:1" ht="26.4">
       <c r="A4" s="7" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="16" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="18" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -1295,27 +1329,27 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="C1" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="16" t="s">
-        <v>132</v>
+      <c r="D1" s="16" t="s">
+        <v>161</v>
       </c>
-      <c r="C1" s="17" t="s">
+    </row>
+    <row r="2" spans="1:4">
+      <c r="C2" s="3"/>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="D1" s="16" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="C2" s="3"/>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="16" t="s">
+      <c r="B4" s="16" t="s">
         <v>135</v>
-      </c>
-      <c r="B4" s="16" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1357,13 +1391,13 @@
   <sheetData>
     <row r="1" spans="1:13">
       <c r="A1" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D1" s="16" t="s">
         <v>2</v>
@@ -1372,28 +1406,28 @@
         <v>0</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G1" s="16" t="s">
         <v>1</v>
       </c>
       <c r="H1" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="J1" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="J1" s="16" t="s">
+      <c r="K1" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="L1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="16" t="s">
         <v>16</v>
-      </c>
-      <c r="M1" s="16" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -1418,21 +1452,21 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>Admin!$C$2:$C$37</xm:f>
+            <xm:f>Admin!$E$2:$E$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>J2:J3000</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>Admin!$C$2:$C$38</xm:f>
           </x14:formula1>
           <xm:sqref>G2:G3000</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>Admin!$D$2:$D$55</xm:f>
+            <xm:f>Admin!$D$2:$D$66</xm:f>
           </x14:formula1>
           <xm:sqref>I2:I3000</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>Admin!$E$2:$E$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>J2:J3000</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1453,13 +1487,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="16" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1487,7 +1521,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C1" s="17" t="s">
         <v>6</v>
@@ -27881,7 +27915,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>Admin!$F$2:$F$9</xm:f>
+            <xm:f>Admin!$F$2:$F$8</xm:f>
           </x14:formula1>
           <xm:sqref>C2:C3000</xm:sqref>
         </x14:dataValidation>
@@ -27893,7 +27927,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr defaultRowHeight="13.2"/>
   <cols>
     <col min="1" max="1" width="31.6640625" style="5" bestFit="1" customWidth="1"/>
@@ -27912,16 +27946,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C1" s="14" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E1" s="14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F1" s="15" t="s">
         <v>6</v>
@@ -27934,179 +27968,176 @@
         <v>3</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C2" s="10" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="12" t="s">
-        <v>24</v>
-      </c>
       <c r="E2" s="10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F2" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G2" s="10"/>
       <c r="H2" s="10"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="B3" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>141</v>
-      </c>
       <c r="F3" s="10" t="s">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="G3" s="10"/>
       <c r="H3" s="10"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C4" s="10" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="12" t="s">
-        <v>34</v>
-      </c>
       <c r="E4" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>35</v>
+        <v>143</v>
       </c>
       <c r="G4" s="10"/>
       <c r="H4" s="10"/>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B5" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="D5" s="12" t="s">
         <v>38</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>39</v>
       </c>
       <c r="E5" s="10"/>
       <c r="F5" s="10" t="s">
-        <v>144</v>
+        <v>25</v>
       </c>
       <c r="G5" s="10"/>
       <c r="H5" s="10"/>
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E6" s="10"/>
       <c r="F6" s="10" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="G6" s="10"/>
       <c r="H6" s="10"/>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="G7" s="10"/>
       <c r="H7" s="10"/>
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E8" s="10"/>
       <c r="F8" s="10" t="s">
-        <v>51</v>
+        <v>147</v>
       </c>
       <c r="G8" s="10"/>
       <c r="H8" s="10"/>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>147</v>
-      </c>
       <c r="C9" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E9" s="10"/>
-      <c r="F9" s="10" t="s">
-        <v>148</v>
-      </c>
       <c r="G9" s="10"/>
       <c r="H9" s="10"/>
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="10"/>
@@ -28116,13 +28147,13 @@
     <row r="11" spans="1:8">
       <c r="A11" s="10"/>
       <c r="B11" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E11" s="10"/>
       <c r="F11" s="10"/>
@@ -28132,13 +28163,13 @@
     <row r="12" spans="1:8">
       <c r="A12" s="13"/>
       <c r="B12" s="11" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E12" s="10"/>
       <c r="F12" s="10"/>
@@ -28148,13 +28179,13 @@
     <row r="13" spans="1:8">
       <c r="A13" s="10"/>
       <c r="B13" s="11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E13" s="10"/>
       <c r="F13" s="10"/>
@@ -28164,13 +28195,13 @@
     <row r="14" spans="1:8">
       <c r="A14" s="10"/>
       <c r="B14" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E14" s="10"/>
       <c r="F14" s="10"/>
@@ -28180,13 +28211,13 @@
     <row r="15" spans="1:8">
       <c r="A15" s="10"/>
       <c r="B15" s="11" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="10"/>
@@ -28196,13 +28227,13 @@
     <row r="16" spans="1:8">
       <c r="A16" s="10"/>
       <c r="B16" s="11" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E16" s="10"/>
       <c r="F16" s="10"/>
@@ -28212,13 +28243,13 @@
     <row r="17" spans="1:8">
       <c r="A17" s="10"/>
       <c r="B17" s="11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E17" s="10"/>
       <c r="F17" s="10"/>
@@ -28228,13 +28259,13 @@
     <row r="18" spans="1:8">
       <c r="A18" s="10"/>
       <c r="B18" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E18" s="10"/>
       <c r="F18" s="10"/>
@@ -28244,13 +28275,13 @@
     <row r="19" spans="1:8">
       <c r="A19" s="10"/>
       <c r="B19" s="11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
@@ -28260,13 +28291,13 @@
     <row r="20" spans="1:8">
       <c r="A20" s="10"/>
       <c r="B20" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D20" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
@@ -28276,13 +28307,13 @@
     <row r="21" spans="1:8">
       <c r="A21" s="10"/>
       <c r="B21" s="11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
@@ -28292,13 +28323,13 @@
     <row r="22" spans="1:8">
       <c r="A22" s="10"/>
       <c r="B22" s="11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>154</v>
+        <v>177</v>
       </c>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
@@ -28308,13 +28339,13 @@
     <row r="23" spans="1:8">
       <c r="A23" s="10"/>
       <c r="B23" s="11" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C23" s="10" t="s">
         <v>4</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
@@ -28324,13 +28355,13 @@
     <row r="24" spans="1:8">
       <c r="A24" s="10"/>
       <c r="B24" s="11" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
@@ -28340,13 +28371,13 @@
     <row r="25" spans="1:8">
       <c r="A25" s="10"/>
       <c r="B25" s="11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
@@ -28356,13 +28387,13 @@
     <row r="26" spans="1:8">
       <c r="A26" s="10"/>
       <c r="B26" s="11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D26" s="10" t="s">
-        <v>73</v>
+        <v>165</v>
       </c>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
@@ -28372,13 +28403,13 @@
     <row r="27" spans="1:8">
       <c r="A27" s="10"/>
       <c r="B27" s="11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>76</v>
+        <v>166</v>
       </c>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
@@ -28388,13 +28419,13 @@
     <row r="28" spans="1:8">
       <c r="A28" s="10"/>
       <c r="B28" s="11" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
@@ -28404,13 +28435,13 @@
     <row r="29" spans="1:8">
       <c r="A29" s="10"/>
       <c r="B29" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
@@ -28420,13 +28451,13 @@
     <row r="30" spans="1:8">
       <c r="A30" s="10"/>
       <c r="B30" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="C30" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="C30" s="10" t="s">
-        <v>89</v>
-      </c>
       <c r="D30" s="10" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
@@ -28437,10 +28468,10 @@
       <c r="A31" s="10"/>
       <c r="B31" s="11"/>
       <c r="C31" s="10" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="E31" s="10"/>
       <c r="F31" s="10"/>
@@ -28450,11 +28481,11 @@
     <row r="32" spans="1:8">
       <c r="A32" s="10"/>
       <c r="B32" s="11"/>
-      <c r="C32" s="10" t="s">
-        <v>93</v>
+      <c r="C32" s="5" t="s">
+        <v>164</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
@@ -28465,10 +28496,10 @@
       <c r="A33" s="10"/>
       <c r="B33" s="11"/>
       <c r="C33" s="10" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
@@ -28479,10 +28510,10 @@
       <c r="A34" s="10"/>
       <c r="B34" s="11"/>
       <c r="C34" s="10" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="D34" s="10" t="s">
-        <v>125</v>
+        <v>89</v>
       </c>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
@@ -28496,7 +28527,7 @@
         <v>118</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>126</v>
+        <v>91</v>
       </c>
       <c r="E35" s="10"/>
       <c r="F35" s="10"/>
@@ -28507,10 +28538,10 @@
       <c r="A36" s="10"/>
       <c r="B36" s="11"/>
       <c r="C36" s="10" t="s">
-        <v>160</v>
+        <v>117</v>
       </c>
       <c r="D36" s="10" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E36" s="10"/>
       <c r="F36" s="10"/>
@@ -28521,10 +28552,10 @@
       <c r="A37" s="10"/>
       <c r="B37" s="10"/>
       <c r="C37" s="10" t="s">
-        <v>46</v>
+        <v>157</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="E37" s="10"/>
       <c r="F37" s="10"/>
@@ -28534,9 +28565,11 @@
     <row r="38" spans="1:8">
       <c r="A38" s="10"/>
       <c r="B38" s="10"/>
-      <c r="C38" s="10"/>
+      <c r="C38" s="10" t="s">
+        <v>45</v>
+      </c>
       <c r="D38" s="10" t="s">
-        <v>98</v>
+        <v>126</v>
       </c>
       <c r="E38" s="10"/>
       <c r="F38" s="10"/>
@@ -28548,7 +28581,7 @@
       <c r="B39" s="11"/>
       <c r="C39" s="10"/>
       <c r="D39" s="10" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="E39" s="10"/>
       <c r="F39" s="10"/>
@@ -28560,7 +28593,7 @@
       <c r="B40" s="11"/>
       <c r="C40" s="10"/>
       <c r="D40" s="10" t="s">
-        <v>129</v>
+        <v>168</v>
       </c>
       <c r="E40" s="10"/>
       <c r="F40" s="10"/>
@@ -28569,77 +28602,132 @@
     </row>
     <row r="41" spans="1:8">
       <c r="D41" s="5" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="D42" s="5" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="D43" s="5" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="D44" s="5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="D45" s="10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="D46" s="10" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="D47" s="10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="D48" s="5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="49" spans="4:4">
+      <c r="D49" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="50" spans="4:4">
+      <c r="D50" s="5" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
-      <c r="D42" s="5" t="s">
+    <row r="51" spans="4:4">
+      <c r="D51" s="5" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="52" spans="4:4">
+      <c r="D52" s="5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="53" spans="4:4">
+      <c r="D53" s="5" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="54" spans="4:4">
+      <c r="D54" s="5" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="55" spans="4:4">
+      <c r="D55" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="56" spans="4:4">
+      <c r="D56" s="5" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
-      <c r="D43" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8">
-      <c r="D44" s="5" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8">
-      <c r="D45" s="5" t="s">
+    <row r="57" spans="4:4">
+      <c r="D57" s="5" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
-      <c r="D46" s="5" t="s">
+    <row r="58" spans="4:4">
+      <c r="D58" s="5" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
-      <c r="D47" s="5" t="s">
+    <row r="59" spans="4:4">
+      <c r="D59" s="5" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
-      <c r="D48" s="5" t="s">
+    <row r="60" spans="4:4">
+      <c r="D60" s="5" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="49" spans="4:4">
-      <c r="D49" s="5" t="s">
+    <row r="61" spans="4:4">
+      <c r="D61" s="5" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="50" spans="4:4">
-      <c r="D50" s="5" t="s">
+    <row r="62" spans="4:4">
+      <c r="D62" s="5" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="51" spans="4:4">
-      <c r="D51" s="5" t="s">
-        <v>108</v>
+    <row r="63" spans="4:4">
+      <c r="D63" s="5" t="s">
+        <v>95</v>
       </c>
     </row>
-    <row r="52" spans="4:4">
-      <c r="D52" s="5" t="s">
+    <row r="64" spans="4:4">
+      <c r="D64" s="5" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="53" spans="4:4">
-      <c r="D53" s="5" t="s">
-        <v>97</v>
+    <row r="65" spans="4:4">
+      <c r="D65" s="5" t="s">
+        <v>127</v>
       </c>
     </row>
-    <row r="54" spans="4:4">
-      <c r="D54" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="55" spans="4:4">
-      <c r="D55" s="5" t="s">
-        <v>88</v>
+    <row r="66" spans="4:4">
+      <c r="D66" s="5" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>